<commit_message>
Added Validation of Obv list with Master list
</commit_message>
<xml_diff>
--- a/Populated_MTC.xlsx
+++ b/Populated_MTC.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="23260" windowHeight="12460" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="hrd" sheetId="1" state="visible" r:id="rId1"/>
@@ -854,32 +854,61 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="29">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="27">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="29">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="29">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -887,9 +916,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="29">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -911,59 +937,33 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="29">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="29">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="27">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="27">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="15">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1326,9 +1326,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1366,9 +1366,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1401,26 +1401,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1453,26 +1436,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1651,20 +1617,20 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:BS33"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="3.6640625" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="3.6640625" defaultRowHeight="16"/>
   <cols>
-    <col width="5.88671875" customWidth="1" style="3" min="1" max="1"/>
-    <col width="18.44140625" customWidth="1" style="3" min="2" max="2"/>
-    <col width="16.44140625" customWidth="1" style="3" min="3" max="3"/>
-    <col width="4.44140625" customWidth="1" style="3" min="4" max="36"/>
-    <col width="26.88671875" customWidth="1" style="3" min="37" max="37"/>
+    <col width="5.83203125" customWidth="1" style="3" min="1" max="1"/>
+    <col width="18.5" customWidth="1" style="3" min="2" max="2"/>
+    <col width="16.5" customWidth="1" style="3" min="3" max="3"/>
+    <col width="4.5" customWidth="1" style="3" min="4" max="36"/>
+    <col width="26.83203125" customWidth="1" style="3" min="37" max="37"/>
     <col width="16.6640625" customWidth="1" style="4" min="38" max="38"/>
-    <col width="12.44140625" customWidth="1" style="4" min="39" max="71"/>
+    <col width="12.5" customWidth="1" style="4" min="39" max="71"/>
     <col width="3.6640625" customWidth="1" style="3" min="72" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="43" t="n"/>
+      <c r="A1" s="19" t="n"/>
       <c r="B1" s="59" t="n"/>
       <c r="C1" s="60" t="n"/>
       <c r="D1" s="61" t="inlineStr">
@@ -1696,14 +1662,14 @@
       <c r="Z1" s="59" t="n"/>
       <c r="AA1" s="59" t="n"/>
       <c r="AB1" s="59" t="n"/>
-      <c r="AC1" s="23" t="inlineStr">
+      <c r="AC1" s="50" t="inlineStr">
         <is>
           <t>Format No.</t>
         </is>
       </c>
       <c r="AD1" s="62" t="n"/>
       <c r="AE1" s="63" t="n"/>
-      <c r="AF1" s="24" t="inlineStr">
+      <c r="AF1" s="51" t="inlineStr">
         <is>
           <t>:QC/F/36/REV. 03</t>
         </is>
@@ -1752,14 +1718,14 @@
       <c r="A2" s="64" t="n"/>
       <c r="C2" s="65" t="n"/>
       <c r="D2" s="64" t="n"/>
-      <c r="AC2" s="23" t="inlineStr">
+      <c r="AC2" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Document No. </t>
         </is>
       </c>
       <c r="AD2" s="62" t="n"/>
       <c r="AE2" s="63" t="n"/>
-      <c r="AF2" s="24" t="n"/>
+      <c r="AF2" s="51" t="n"/>
       <c r="AG2" s="62" t="n"/>
       <c r="AH2" s="62" t="n"/>
       <c r="AI2" s="62" t="n"/>
@@ -1828,14 +1794,14 @@
       <c r="Z3" s="67" t="n"/>
       <c r="AA3" s="67" t="n"/>
       <c r="AB3" s="67" t="n"/>
-      <c r="AC3" s="23" t="inlineStr">
+      <c r="AC3" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Revision </t>
         </is>
       </c>
       <c r="AD3" s="62" t="n"/>
       <c r="AE3" s="63" t="n"/>
-      <c r="AF3" s="24" t="n"/>
+      <c r="AF3" s="51" t="n"/>
       <c r="AG3" s="62" t="n"/>
       <c r="AH3" s="62" t="n"/>
       <c r="AI3" s="62" t="n"/>
@@ -1879,7 +1845,7 @@
     <row r="4" ht="18.75" customHeight="1">
       <c r="A4" s="64" t="n"/>
       <c r="C4" s="65" t="n"/>
-      <c r="D4" s="51" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>KINGDOM OF SAUDI ARABIA</t>
         </is>
@@ -1908,7 +1874,7 @@
       <c r="Z4" s="67" t="n"/>
       <c r="AA4" s="67" t="n"/>
       <c r="AB4" s="67" t="n"/>
-      <c r="AC4" s="23" t="inlineStr">
+      <c r="AC4" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Date  </t>
         </is>
@@ -1960,7 +1926,7 @@
       <c r="A5" s="66" t="n"/>
       <c r="B5" s="67" t="n"/>
       <c r="C5" s="69" t="n"/>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="D5" s="29" t="inlineStr">
         <is>
           <t>QUALITY CONTROL</t>
         </is>
@@ -1989,14 +1955,14 @@
       <c r="Z5" s="62" t="n"/>
       <c r="AA5" s="62" t="n"/>
       <c r="AB5" s="62" t="n"/>
-      <c r="AC5" s="23" t="inlineStr">
+      <c r="AC5" s="50" t="inlineStr">
         <is>
           <t>Pages</t>
         </is>
       </c>
       <c r="AD5" s="62" t="n"/>
       <c r="AE5" s="63" t="n"/>
-      <c r="AF5" s="24" t="n"/>
+      <c r="AF5" s="51" t="n"/>
       <c r="AG5" s="62" t="n"/>
       <c r="AH5" s="62" t="n"/>
       <c r="AI5" s="62" t="n"/>
@@ -2038,14 +2004,14 @@
       <c r="BS5" s="3" t="n"/>
     </row>
     <row r="6" ht="18.75" customHeight="1">
-      <c r="A6" s="55" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>Document</t>
         </is>
       </c>
       <c r="B6" s="62" t="n"/>
       <c r="C6" s="63" t="n"/>
-      <c r="D6" s="53" t="inlineStr">
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>MILL TEST CERTIFICATE (AS PER BS EN 10204:2004 TYPE 3.1)</t>
         </is>
@@ -2074,14 +2040,14 @@
       <c r="Z6" s="62" t="n"/>
       <c r="AA6" s="62" t="n"/>
       <c r="AB6" s="62" t="n"/>
-      <c r="AC6" s="23" t="inlineStr">
+      <c r="AC6" s="50" t="inlineStr">
         <is>
           <t>Annexure No.</t>
         </is>
       </c>
       <c r="AD6" s="62" t="n"/>
       <c r="AE6" s="63" t="n"/>
-      <c r="AF6" s="24" t="n"/>
+      <c r="AF6" s="51" t="n"/>
       <c r="AG6" s="62" t="n"/>
       <c r="AH6" s="62" t="n"/>
       <c r="AI6" s="62" t="n"/>
@@ -2123,18 +2089,18 @@
       <c r="BS6" s="3" t="n"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="57" t="inlineStr">
+      <c r="A7" s="35" t="inlineStr">
         <is>
           <t>MANUFACTURER</t>
         </is>
       </c>
-      <c r="C7" s="42" t="n"/>
-      <c r="N7" s="30" t="inlineStr">
+      <c r="C7" s="32" t="n"/>
+      <c r="N7" s="37" t="inlineStr">
         <is>
           <t>ITP No.</t>
         </is>
       </c>
-      <c r="Q7" s="30" t="n"/>
+      <c r="Q7" s="37" t="n"/>
       <c r="AC7" s="7" t="n"/>
       <c r="AD7" s="1" t="n"/>
       <c r="AE7" s="1" t="n"/>
@@ -2146,12 +2112,12 @@
       <c r="AK7" s="12" t="n"/>
     </row>
     <row r="8" ht="34.5" customHeight="1">
-      <c r="A8" s="57" t="inlineStr">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>CLIENT</t>
         </is>
       </c>
-      <c r="C8" s="42" t="n"/>
+      <c r="C8" s="32" t="n"/>
       <c r="AC8" s="7" t="n"/>
       <c r="AD8" s="1" t="n"/>
       <c r="AE8" s="1" t="n"/>
@@ -2164,12 +2130,12 @@
       <c r="AL8" s="2" t="n"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="41" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>PROJECT</t>
         </is>
       </c>
-      <c r="C9" s="42" t="n"/>
+      <c r="C9" s="32" t="n"/>
       <c r="AC9" s="7" t="n"/>
       <c r="AD9" s="1" t="n"/>
       <c r="AE9" s="1" t="n"/>
@@ -2181,12 +2147,12 @@
       <c r="AK9" s="12" t="n"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="38" t="inlineStr">
         <is>
           <t>P. O. NO.</t>
         </is>
       </c>
-      <c r="C10" s="30" t="n"/>
+      <c r="C10" s="37" t="n"/>
       <c r="AC10" s="8" t="n"/>
       <c r="AD10" s="1" t="n"/>
       <c r="AE10" s="1" t="n"/>
@@ -2198,12 +2164,12 @@
       <c r="AK10" s="12" t="n"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>PIPE SIZE / MATERIAL SPEC.</t>
         </is>
       </c>
-      <c r="C11" s="30" t="n"/>
+      <c r="C11" s="37" t="n"/>
       <c r="AC11" s="7" t="n"/>
       <c r="AD11" s="1" t="n"/>
       <c r="AE11" s="1" t="n"/>
@@ -2215,12 +2181,12 @@
       <c r="AK11" s="12" t="n"/>
     </row>
     <row r="12" ht="48.75" customHeight="1">
-      <c r="A12" s="41" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>MFG./TECHNICAL SPECIFICATION</t>
         </is>
       </c>
-      <c r="C12" s="42" t="n"/>
+      <c r="C12" s="32" t="n"/>
       <c r="AC12" s="7" t="n"/>
       <c r="AD12" s="1" t="n"/>
       <c r="AE12" s="1" t="n"/>
@@ -2282,15 +2248,15 @@
       </c>
       <c r="B14" s="70" t="inlineStr">
         <is>
+          <t>PIPE NO.</t>
+        </is>
+      </c>
+      <c r="C14" s="70" t="inlineStr">
+        <is>
           <t>HEAT NO.</t>
         </is>
       </c>
-      <c r="C14" s="70" t="inlineStr">
-        <is>
-          <t>PIPE NO.</t>
-        </is>
-      </c>
-      <c r="D14" s="37" t="inlineStr">
+      <c r="D14" s="46" t="inlineStr">
         <is>
           <t>CORRESPONDING HARDNESS VALUES AT HV10</t>
         </is>
@@ -2369,7 +2335,7 @@
       <c r="Y15" s="62" t="n"/>
       <c r="Z15" s="62" t="n"/>
       <c r="AA15" s="63" t="n"/>
-      <c r="AB15" s="31" t="inlineStr">
+      <c r="AB15" s="40" t="inlineStr">
         <is>
           <t>WELD</t>
         </is>
@@ -2484,7 +2450,7 @@
       <c r="AI16" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="AJ16" s="31" t="n">
+      <c r="AJ16" s="40" t="n">
         <v>33</v>
       </c>
       <c r="AK16" s="72" t="n"/>
@@ -2500,11 +2466,11 @@
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>2601251</t>
+          <t>260125.3</t>
         </is>
       </c>
       <c r="D17" s="15" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E17" s="15" t="n">
         <v>188</v>
@@ -2561,7 +2527,7 @@
         <v>164</v>
       </c>
       <c r="W17" s="15" t="n">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="X17" s="15" t="n">
         <v>181</v>
@@ -2619,11 +2585,11 @@
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>2601235</t>
+          <t>260123.5</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E18" s="15" t="n">
         <v>191</v>
@@ -2710,7 +2676,7 @@
         <v>204</v>
       </c>
       <c r="AG18" s="15" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AH18" s="15" t="n">
         <v>199</v>
@@ -2738,7 +2704,7 @@
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>2551275</t>
+          <t>255127.5</t>
         </is>
       </c>
       <c r="D19" s="15" t="n">
@@ -2842,7 +2808,7 @@
       </c>
       <c r="AK19" s="18" t="inlineStr">
         <is>
-          <t>HEAT-T</t>
+          <t>HEAT</t>
         </is>
       </c>
     </row>
@@ -2857,11 +2823,11 @@
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>2552316</t>
+          <t>255231.6</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E20" s="15" t="n">
         <v>192</v>
@@ -2930,7 +2896,7 @@
         <v>176</v>
       </c>
       <c r="AA20" s="15" t="n">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="AB20" s="15" t="n">
         <v>201</v>
@@ -3200,7 +3166,7 @@
       <c r="AK26" s="18" t="n"/>
     </row>
     <row r="27" ht="32.25" customHeight="1">
-      <c r="A27" s="22" t="inlineStr">
+      <c r="A27" s="55" t="inlineStr">
         <is>
           <t>NOTE: INDENTATION POINT FOR BASE METAL ARE 1 to 6, INDENTATION POINT FOR HAZ ARE 7 to 24 &amp; INDENTATION POINT FOR WELD METAL ARE 25 to 33. Hardness indentation as per figure H.1 in API 5L and clause SAMSS 035 H.7.3.3.3</t>
         </is>
@@ -3243,7 +3209,7 @@
       <c r="AK27" s="74" t="n"/>
     </row>
     <row r="28" ht="24.75" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="56" t="inlineStr">
         <is>
           <t>PREPARED BY:</t>
         </is>
@@ -3252,7 +3218,7 @@
       <c r="C28" s="62" t="n"/>
       <c r="D28" s="62" t="n"/>
       <c r="E28" s="63" t="n"/>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="F28" s="56" t="inlineStr">
         <is>
           <t>REVIEWED BY:</t>
         </is>
@@ -3268,7 +3234,7 @@
       <c r="O28" s="62" t="n"/>
       <c r="P28" s="62" t="n"/>
       <c r="Q28" s="63" t="n"/>
-      <c r="R28" s="21" t="inlineStr">
+      <c r="R28" s="56" t="inlineStr">
         <is>
           <t>APPROVED BY:</t>
         </is>
@@ -3284,7 +3250,7 @@
       <c r="AA28" s="62" t="n"/>
       <c r="AB28" s="62" t="n"/>
       <c r="AC28" s="63" t="n"/>
-      <c r="AD28" s="21" t="inlineStr">
+      <c r="AD28" s="56" t="inlineStr">
         <is>
           <t>CLIENT/TPI APPROVAL</t>
         </is>
@@ -3298,12 +3264,12 @@
       <c r="AK28" s="63" t="n"/>
     </row>
     <row r="29" ht="26.25" customHeight="1">
-      <c r="A29" s="20" t="n"/>
+      <c r="A29" s="58" t="n"/>
       <c r="B29" s="59" t="n"/>
       <c r="C29" s="59" t="n"/>
       <c r="D29" s="59" t="n"/>
       <c r="E29" s="60" t="n"/>
-      <c r="F29" s="21" t="n"/>
+      <c r="F29" s="56" t="n"/>
       <c r="G29" s="59" t="n"/>
       <c r="H29" s="59" t="n"/>
       <c r="I29" s="59" t="n"/>
@@ -3315,7 +3281,7 @@
       <c r="O29" s="59" t="n"/>
       <c r="P29" s="59" t="n"/>
       <c r="Q29" s="60" t="n"/>
-      <c r="R29" s="21" t="n"/>
+      <c r="R29" s="56" t="n"/>
       <c r="S29" s="59" t="n"/>
       <c r="T29" s="59" t="n"/>
       <c r="U29" s="59" t="n"/>
@@ -3327,7 +3293,7 @@
       <c r="AA29" s="59" t="n"/>
       <c r="AB29" s="59" t="n"/>
       <c r="AC29" s="60" t="n"/>
-      <c r="AD29" s="21" t="n"/>
+      <c r="AD29" s="56" t="n"/>
       <c r="AE29" s="59" t="n"/>
       <c r="AF29" s="59" t="n"/>
       <c r="AG29" s="59" t="n"/>
@@ -3386,7 +3352,7 @@
       <c r="AK31" s="69" t="n"/>
     </row>
     <row r="32" ht="24.75" customHeight="1">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="57" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
@@ -3395,7 +3361,7 @@
       <c r="C32" s="62" t="n"/>
       <c r="D32" s="62" t="n"/>
       <c r="E32" s="63" t="n"/>
-      <c r="F32" s="19" t="inlineStr">
+      <c r="F32" s="57" t="inlineStr">
         <is>
           <t>LAB IN CHARGE</t>
         </is>
@@ -3411,7 +3377,7 @@
       <c r="O32" s="62" t="n"/>
       <c r="P32" s="62" t="n"/>
       <c r="Q32" s="63" t="n"/>
-      <c r="R32" s="19" t="inlineStr">
+      <c r="R32" s="57" t="inlineStr">
         <is>
           <t>HEAD QUALITY &amp; TS</t>
         </is>
@@ -3427,7 +3393,7 @@
       <c r="AA32" s="62" t="n"/>
       <c r="AB32" s="62" t="n"/>
       <c r="AC32" s="63" t="n"/>
-      <c r="AD32" s="19" t="inlineStr">
+      <c r="AD32" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">SA VID / SA VID REPRESENTATIVE </t>
         </is>
@@ -3441,7 +3407,7 @@
       <c r="AK32" s="63" t="n"/>
     </row>
     <row r="33" ht="24.75" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="57" t="inlineStr">
         <is>
           <t>BENJAMIN BON</t>
         </is>
@@ -3450,7 +3416,7 @@
       <c r="C33" s="62" t="n"/>
       <c r="D33" s="62" t="n"/>
       <c r="E33" s="63" t="n"/>
-      <c r="F33" s="19" t="inlineStr">
+      <c r="F33" s="57" t="inlineStr">
         <is>
           <t>MOSTAFA SARSAK</t>
         </is>
@@ -3466,7 +3432,7 @@
       <c r="O33" s="62" t="n"/>
       <c r="P33" s="62" t="n"/>
       <c r="Q33" s="63" t="n"/>
-      <c r="R33" s="19" t="inlineStr">
+      <c r="R33" s="57" t="inlineStr">
         <is>
           <t>DHAVAL VORA</t>
         </is>
@@ -3482,7 +3448,7 @@
       <c r="AA33" s="62" t="n"/>
       <c r="AB33" s="62" t="n"/>
       <c r="AC33" s="63" t="n"/>
-      <c r="AD33" s="19" t="inlineStr">
+      <c r="AD33" s="57" t="inlineStr">
         <is>
           <t>HITESH KUMAR JAIN - APPLUS VELOSI</t>
         </is>
@@ -3501,13 +3467,13 @@
     <mergeCell ref="AC5:AE5"/>
     <mergeCell ref="J15:AA15"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="F33:Q33"/>
     <mergeCell ref="D4:AB4"/>
-    <mergeCell ref="F33:Q33"/>
     <mergeCell ref="AF6:AK6"/>
     <mergeCell ref="AD33:AK33"/>
     <mergeCell ref="F32:Q32"/>
+    <mergeCell ref="AC4:AE4"/>
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="AC4:AE4"/>
     <mergeCell ref="AC1:AE1"/>
     <mergeCell ref="AF2:AK2"/>
     <mergeCell ref="A7:B7"/>
@@ -3516,8 +3482,8 @@
     <mergeCell ref="D5:AB5"/>
     <mergeCell ref="R32:AC32"/>
     <mergeCell ref="AD29:AK31"/>
+    <mergeCell ref="AD28:AK28"/>
     <mergeCell ref="D1:AB3"/>
-    <mergeCell ref="AD28:AK28"/>
     <mergeCell ref="C10:AB10"/>
     <mergeCell ref="AC6:AE6"/>
     <mergeCell ref="D15:I15"/>
@@ -3531,35 +3497,35 @@
     <mergeCell ref="C12:AB12"/>
     <mergeCell ref="A32:E32"/>
     <mergeCell ref="AF3:AK3"/>
+    <mergeCell ref="D6:AB6"/>
+    <mergeCell ref="AD32:AK32"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="D6:AB6"/>
-    <mergeCell ref="Q7:AB7"/>
     <mergeCell ref="C11:AB11"/>
     <mergeCell ref="D14:AJ14"/>
-    <mergeCell ref="AD32:AK32"/>
+    <mergeCell ref="Q7:AB7"/>
     <mergeCell ref="AB15:AJ15"/>
+    <mergeCell ref="AK14:AK16"/>
     <mergeCell ref="N7:P7"/>
-    <mergeCell ref="AK14:AK16"/>
     <mergeCell ref="F29:Q31"/>
+    <mergeCell ref="A29:E31"/>
     <mergeCell ref="C8:AB8"/>
-    <mergeCell ref="A29:E31"/>
     <mergeCell ref="C7:M7"/>
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="R29:AC31"/>
+    <mergeCell ref="A10:B10"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="R28:AC28"/>
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="R28:AC28"/>
     <mergeCell ref="AC3:AE3"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A27:AK27"/>
     <mergeCell ref="AF4:AK4"/>
   </mergeCells>
+  <conditionalFormatting sqref="B1:B16 B34:B1048576">
+    <cfRule type="duplicateValues" priority="180" dxfId="0"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" priority="1" dxfId="0"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B16 B34:B1048576">
-    <cfRule type="duplicateValues" priority="180" dxfId="0"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:B33">
     <cfRule type="duplicateValues" priority="183" dxfId="0"/>

</xml_diff>